<commit_message>
fixed sensedComponent excel output
</commit_message>
<xml_diff>
--- a/shipClassTests/testResults/comp_test.xlsx
+++ b/shipClassTests/testResults/comp_test.xlsx
@@ -561,7 +561,7 @@
         <v>19</v>
       </c>
       <c r="B21" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22" spans="1:2">
@@ -569,7 +569,7 @@
         <v>20</v>
       </c>
       <c r="B22" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -577,7 +577,7 @@
         <v>21</v>
       </c>
       <c r="B23" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24" spans="1:2">
@@ -585,7 +585,7 @@
         <v>22</v>
       </c>
       <c r="B24" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25" spans="1:2">
@@ -593,7 +593,7 @@
         <v>23</v>
       </c>
       <c r="B25" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:2">
@@ -601,7 +601,7 @@
         <v>24</v>
       </c>
       <c r="B26" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:2">
@@ -609,7 +609,7 @@
         <v>25</v>
       </c>
       <c r="B27" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:2">
@@ -617,7 +617,7 @@
         <v>26</v>
       </c>
       <c r="B28" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:2">
@@ -625,7 +625,7 @@
         <v>27</v>
       </c>
       <c r="B29" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:2">
@@ -633,7 +633,7 @@
         <v>28</v>
       </c>
       <c r="B30" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:2">
@@ -641,7 +641,7 @@
         <v>29</v>
       </c>
       <c r="B31" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:2">
@@ -649,7 +649,7 @@
         <v>30</v>
       </c>
       <c r="B32" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -657,7 +657,7 @@
         <v>31</v>
       </c>
       <c r="B33" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -665,7 +665,7 @@
         <v>32</v>
       </c>
       <c r="B34" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:2">
@@ -673,7 +673,7 @@
         <v>33</v>
       </c>
       <c r="B35" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36" spans="1:2">
@@ -681,7 +681,7 @@
         <v>34</v>
       </c>
       <c r="B36" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:2">
@@ -689,7 +689,7 @@
         <v>35</v>
       </c>
       <c r="B37" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:2">
@@ -697,7 +697,7 @@
         <v>36</v>
       </c>
       <c r="B38" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:2">
@@ -705,7 +705,7 @@
         <v>37</v>
       </c>
       <c r="B39" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:2">
@@ -713,7 +713,7 @@
         <v>38</v>
       </c>
       <c r="B40" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41" spans="1:2">
@@ -721,7 +721,7 @@
         <v>39</v>
       </c>
       <c r="B41" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42" spans="1:2">
@@ -729,7 +729,7 @@
         <v>40</v>
       </c>
       <c r="B42" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -737,7 +737,7 @@
         <v>41</v>
       </c>
       <c r="B43" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -745,7 +745,7 @@
         <v>42</v>
       </c>
       <c r="B44" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -753,7 +753,7 @@
         <v>43</v>
       </c>
       <c r="B45" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -761,7 +761,7 @@
         <v>44</v>
       </c>
       <c r="B46" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -769,7 +769,7 @@
         <v>45</v>
       </c>
       <c r="B47" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -777,7 +777,7 @@
         <v>46</v>
       </c>
       <c r="B48" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -785,7 +785,7 @@
         <v>47</v>
       </c>
       <c r="B49" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -793,7 +793,7 @@
         <v>48</v>
       </c>
       <c r="B50" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51" spans="1:2">
@@ -801,7 +801,7 @@
         <v>49</v>
       </c>
       <c r="B51" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -809,7 +809,7 @@
         <v>50</v>
       </c>
       <c r="B52" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53" spans="1:2">
@@ -817,7 +817,7 @@
         <v>51</v>
       </c>
       <c r="B53" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -825,7 +825,7 @@
         <v>52</v>
       </c>
       <c r="B54" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55" spans="1:2">
@@ -833,7 +833,7 @@
         <v>53</v>
       </c>
       <c r="B55" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56" spans="1:2">
@@ -841,7 +841,7 @@
         <v>54</v>
       </c>
       <c r="B56" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57" spans="1:2">
@@ -849,7 +849,7 @@
         <v>55</v>
       </c>
       <c r="B57" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="58" spans="1:2">
@@ -857,7 +857,7 @@
         <v>56</v>
       </c>
       <c r="B58" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="59" spans="1:2">
@@ -865,7 +865,7 @@
         <v>57</v>
       </c>
       <c r="B59" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="60" spans="1:2">
@@ -873,7 +873,7 @@
         <v>58</v>
       </c>
       <c r="B60" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -881,7 +881,7 @@
         <v>59</v>
       </c>
       <c r="B61" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -889,7 +889,7 @@
         <v>60</v>
       </c>
       <c r="B62" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -897,7 +897,7 @@
         <v>61</v>
       </c>
       <c r="B63" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="64" spans="1:2">
@@ -905,7 +905,7 @@
         <v>62</v>
       </c>
       <c r="B64" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="65" spans="1:2">
@@ -913,7 +913,7 @@
         <v>63</v>
       </c>
       <c r="B65" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="66" spans="1:2">
@@ -921,7 +921,7 @@
         <v>64</v>
       </c>
       <c r="B66" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="67" spans="1:2">
@@ -929,7 +929,7 @@
         <v>65</v>
       </c>
       <c r="B67" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="68" spans="1:2">
@@ -937,7 +937,7 @@
         <v>66</v>
       </c>
       <c r="B68" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -945,7 +945,7 @@
         <v>67</v>
       </c>
       <c r="B69" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -953,7 +953,7 @@
         <v>68</v>
       </c>
       <c r="B70" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -961,7 +961,7 @@
         <v>69</v>
       </c>
       <c r="B71" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="72" spans="1:2">
@@ -969,7 +969,7 @@
         <v>70</v>
       </c>
       <c r="B72" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="73" spans="1:2">
@@ -977,7 +977,7 @@
         <v>71</v>
       </c>
       <c r="B73" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="74" spans="1:2">
@@ -985,7 +985,7 @@
         <v>72</v>
       </c>
       <c r="B74" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="75" spans="1:2">
@@ -993,7 +993,7 @@
         <v>73</v>
       </c>
       <c r="B75" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="76" spans="1:2">
@@ -1001,7 +1001,7 @@
         <v>74</v>
       </c>
       <c r="B76" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -1009,7 +1009,7 @@
         <v>75</v>
       </c>
       <c r="B77" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -1017,7 +1017,7 @@
         <v>76</v>
       </c>
       <c r="B78" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="79" spans="1:2">
@@ -1025,7 +1025,7 @@
         <v>77</v>
       </c>
       <c r="B79" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="80" spans="1:2">
@@ -1033,7 +1033,7 @@
         <v>78</v>
       </c>
       <c r="B80" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -1041,7 +1041,7 @@
         <v>79</v>
       </c>
       <c r="B81" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="82" spans="1:2">
@@ -1049,7 +1049,7 @@
         <v>80</v>
       </c>
       <c r="B82" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -1057,7 +1057,7 @@
         <v>81</v>
       </c>
       <c r="B83" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -1065,7 +1065,7 @@
         <v>82</v>
       </c>
       <c r="B84" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -1073,7 +1073,7 @@
         <v>83</v>
       </c>
       <c r="B85" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="86" spans="1:2">
@@ -1081,7 +1081,7 @@
         <v>84</v>
       </c>
       <c r="B86" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="87" spans="1:2">
@@ -1089,7 +1089,7 @@
         <v>85</v>
       </c>
       <c r="B87" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -1097,7 +1097,7 @@
         <v>86</v>
       </c>
       <c r="B88" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -1105,7 +1105,7 @@
         <v>87</v>
       </c>
       <c r="B89" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="90" spans="1:2">
@@ -1113,7 +1113,7 @@
         <v>88</v>
       </c>
       <c r="B90" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="91" spans="1:2">
@@ -1121,7 +1121,7 @@
         <v>89</v>
       </c>
       <c r="B91" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -1129,7 +1129,7 @@
         <v>90</v>
       </c>
       <c r="B92" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="93" spans="1:2">
@@ -1137,7 +1137,7 @@
         <v>91</v>
       </c>
       <c r="B93" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="94" spans="1:2">
@@ -1145,7 +1145,7 @@
         <v>92</v>
       </c>
       <c r="B94" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="95" spans="1:2">
@@ -1153,7 +1153,7 @@
         <v>93</v>
       </c>
       <c r="B95" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="96" spans="1:2">
@@ -1161,7 +1161,7 @@
         <v>94</v>
       </c>
       <c r="B96" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="97" spans="1:2">
@@ -1169,7 +1169,7 @@
         <v>95</v>
       </c>
       <c r="B97" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="98" spans="1:2">
@@ -1177,7 +1177,7 @@
         <v>96</v>
       </c>
       <c r="B98" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="99" spans="1:2">
@@ -1185,7 +1185,7 @@
         <v>97</v>
       </c>
       <c r="B99" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="100" spans="1:2">
@@ -1193,7 +1193,7 @@
         <v>98</v>
       </c>
       <c r="B100" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="101" spans="1:2">
@@ -1201,7 +1201,7 @@
         <v>99</v>
       </c>
       <c r="B101" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="102" spans="1:2">
@@ -1209,7 +1209,7 @@
         <v>100</v>
       </c>
       <c r="B102" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>